<commit_message>
Auto commit 23-06-2025 17:22:00.01
</commit_message>
<xml_diff>
--- a/Templates/ARS Lettering.xlsx
+++ b/Templates/ARS Lettering.xlsx
@@ -1,27 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="120" windowWidth="14940" windowHeight="9225" activeTab="0"/>
+    <workbookView xWindow="240" yWindow="120" windowWidth="14940" windowHeight="9230"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
-  <si>
-    <t>Item Name</t>
-  </si>
-  <si>
-    <t>Quantity</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
   <si>
     <t>Painting with silicon &amp; acrylic emulsion based water thinnable sealer of approved brand and manufacture on wet or patchy portion of plastered surfaces: Two coats (Code: 13.51.2)</t>
   </si>
@@ -32,8 +25,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color theme="1"/>
@@ -65,111 +58,18 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
-      <alignment/>
-      <protection/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Percent" xfId="15" builtinId="5"/>
-    <cellStyle name="Currency" xfId="16" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="17" builtinId="7"/>
-    <cellStyle name="Comma" xfId="18" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="19" builtinId="6"/>
   </cellStyles>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -224,7 +124,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -276,7 +176,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -470,38 +370,30 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F7C65D7-B3D7-48C7-B21E-5E6DE844B9A6}">
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" ht="12.75">
+    <row r="1" spans="1:2" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="1">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" ht="12.75">
-      <c r="A2" s="1" t="s">
-        <v>2</v>
-      </c>
       <c r="B2" s="1">
-        <v>0.80</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="12.75">
-      <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="1">
         <v>250</v>
       </c>
     </row>

</xml_diff>